<commit_message>
fixed weird pad wiring, finished mem/lite v1
</commit_message>
<xml_diff>
--- a/part count estimates.xlsx
+++ b/part count estimates.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc project\rlpc\AX08-PC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEF6C7EE-3337-4BF9-911A-F5CF48A1C542}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDE6CEF4-B448-4F62-AA29-90C248F4C401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="160">
   <si>
     <t>Register File</t>
   </si>
@@ -513,6 +513,12 @@
   </si>
   <si>
     <t>supplements</t>
+  </si>
+  <si>
+    <t>lite + mem</t>
+  </si>
+  <si>
+    <t>PICs, debug</t>
   </si>
 </sst>
 </file>
@@ -2489,7 +2495,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A84AF481-944A-4A4E-812B-EDDAA2A2EDA1}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="8.86328125" customWidth="1"/>
@@ -2511,7 +2517,7 @@
       </c>
       <c r="F1" s="8">
         <f>SUM(C:C)</f>
-        <v>213.29000000000002</v>
+        <v>465.05000000000007</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
@@ -2556,6 +2562,28 @@
       </c>
       <c r="C5" s="4">
         <v>48.95</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B6" t="s">
+        <v>158</v>
+      </c>
+      <c r="C6" s="4">
+        <v>128.54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" t="s">
+        <v>159</v>
+      </c>
+      <c r="C7" s="4">
+        <v>123.22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added my ordered part
</commit_message>
<xml_diff>
--- a/part count estimates.xlsx
+++ b/part count estimates.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc project\rlpc\AX08-PC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projects\computer\ax08\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDE6CEF4-B448-4F62-AA29-90C248F4C401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C39695F-9417-4CDC-B1F3-D23FC2D77ACA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="168">
   <si>
     <t>Register File</t>
   </si>
@@ -519,6 +519,30 @@
   </si>
   <si>
     <t>PICs, debug</t>
+  </si>
+  <si>
+    <t>Buyer</t>
+  </si>
+  <si>
+    <t>Oliver</t>
+  </si>
+  <si>
+    <t>Amazon</t>
+  </si>
+  <si>
+    <t>Netzteile</t>
+  </si>
+  <si>
+    <t>Peter</t>
+  </si>
+  <si>
+    <t>Steckbrett</t>
+  </si>
+  <si>
+    <t>Kabel+Devboards</t>
+  </si>
+  <si>
+    <t>2 x Uart Adapter</t>
   </si>
 </sst>
 </file>
@@ -629,9 +653,9 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Link" xfId="1" builtinId="8"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
-    <cellStyle name="Währung" xfId="2" builtinId="4"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -910,16 +934,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.86328125" customWidth="1"/>
-    <col min="2" max="4" width="10.1328125" customWidth="1"/>
-    <col min="7" max="8" width="10.1328125" customWidth="1"/>
-    <col min="14" max="15" width="10.1328125" customWidth="1"/>
-    <col min="16" max="16" width="48.265625" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" customWidth="1"/>
+    <col min="2" max="4" width="10.140625" customWidth="1"/>
+    <col min="7" max="8" width="10.140625" customWidth="1"/>
+    <col min="14" max="15" width="10.140625" customWidth="1"/>
+    <col min="16" max="16" width="48.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>2</v>
       </c>
@@ -966,7 +990,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1013,7 +1037,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1060,7 +1084,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1107,7 +1131,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -1154,7 +1178,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -1201,7 +1225,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -1248,7 +1272,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1295,7 +1319,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -1342,7 +1366,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -1389,7 +1413,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1439,7 +1463,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>39</v>
       </c>
@@ -1508,14 +1532,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1780C73-0264-4CD0-A807-67CE58F9B4CA}">
   <dimension ref="A1:D36"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.06640625" customWidth="1"/>
-    <col min="2" max="2" width="16.53125" customWidth="1"/>
-    <col min="3" max="3" width="12.73046875" customWidth="1"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="16.5703125" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>129</v>
       </c>
@@ -1529,7 +1553,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>116</v>
       </c>
@@ -1540,7 +1564,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>146</v>
       </c>
@@ -1551,7 +1575,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>119</v>
       </c>
@@ -1562,7 +1586,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>143</v>
       </c>
@@ -1573,7 +1597,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>120</v>
       </c>
@@ -1584,7 +1608,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>121</v>
       </c>
@@ -1595,7 +1619,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>123</v>
       </c>
@@ -1609,7 +1633,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>116</v>
       </c>
@@ -1620,7 +1644,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>119</v>
       </c>
@@ -1631,7 +1655,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>143</v>
       </c>
@@ -1642,7 +1666,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>120</v>
       </c>
@@ -1653,7 +1677,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>130</v>
       </c>
@@ -1667,7 +1691,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>116</v>
       </c>
@@ -1678,7 +1702,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>119</v>
       </c>
@@ -1689,7 +1713,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>143</v>
       </c>
@@ -1700,7 +1724,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>120</v>
       </c>
@@ -1711,7 +1735,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>133</v>
       </c>
@@ -1722,7 +1746,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>134</v>
       </c>
@@ -1733,7 +1757,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>135</v>
       </c>
@@ -1747,7 +1771,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>153</v>
       </c>
@@ -1758,7 +1782,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>150</v>
       </c>
@@ -1769,7 +1793,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>154</v>
       </c>
@@ -1780,7 +1804,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>155</v>
       </c>
@@ -1791,7 +1815,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>156</v>
       </c>
@@ -1802,7 +1826,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>136</v>
       </c>
@@ -1816,7 +1840,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>120</v>
       </c>
@@ -1827,7 +1851,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
         <v>67</v>
       </c>
@@ -1838,7 +1862,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="33" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="33" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
         <v>66</v>
       </c>
@@ -1849,7 +1873,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="34" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="34" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>137</v>
       </c>
@@ -1860,7 +1884,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="35" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="35" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
         <v>138</v>
       </c>
@@ -1871,7 +1895,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="36" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="36" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
         <v>139</v>
       </c>
@@ -1890,14 +1914,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A2F25C3-A040-4D55-A5F0-DFC308DB6F13}">
   <dimension ref="B1:K33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="26.86328125" customWidth="1"/>
-    <col min="3" max="3" width="29.73046875" customWidth="1"/>
-    <col min="6" max="6" width="109.73046875" customWidth="1"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="29.7109375" customWidth="1"/>
+    <col min="6" max="6" width="109.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="H1" t="s">
         <v>35</v>
       </c>
@@ -1909,14 +1933,14 @@
         <v>10.8</v>
       </c>
     </row>
-    <row r="2" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
       <c r="H2" s="4">
         <f>SUM(H5:H996)</f>
         <v>123.93560000000001</v>
       </c>
     </row>
-    <row r="3" spans="2:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="4" spans="2:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="5" t="s">
         <v>28</v>
       </c>
@@ -1935,7 +1959,7 @@
       <c r="G4" s="6"/>
       <c r="H4" s="7"/>
     </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>34</v>
       </c>
@@ -1957,7 +1981,7 @@
         <v>21.6</v>
       </c>
     </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>37</v>
       </c>
@@ -1975,7 +1999,7 @@
         <v>40.599999999999994</v>
       </c>
     </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>40</v>
       </c>
@@ -1996,7 +2020,7 @@
         <v>17.335999999999999</v>
       </c>
     </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>43</v>
       </c>
@@ -2017,7 +2041,7 @@
         <v>7.645999999999999</v>
       </c>
     </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>44</v>
       </c>
@@ -2038,7 +2062,7 @@
         <v>2.7639999999999998</v>
       </c>
     </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>46</v>
       </c>
@@ -2059,7 +2083,7 @@
         <v>1.2089999999999999</v>
       </c>
     </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>51</v>
       </c>
@@ -2080,7 +2104,7 @@
         <v>0.75050000000000006</v>
       </c>
     </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>48</v>
       </c>
@@ -2101,7 +2125,7 @@
         <v>0.9355</v>
       </c>
     </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>53</v>
       </c>
@@ -2122,7 +2146,7 @@
         <v>0.85450000000000004</v>
       </c>
     </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>55</v>
       </c>
@@ -2143,7 +2167,7 @@
         <v>0.7679999999999999</v>
       </c>
     </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>57</v>
       </c>
@@ -2164,7 +2188,7 @@
         <v>1.099</v>
       </c>
     </row>
-    <row r="16" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>59</v>
       </c>
@@ -2185,7 +2209,7 @@
         <v>0.89899999999999991</v>
       </c>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>108</v>
       </c>
@@ -2206,7 +2230,7 @@
         <v>2.0110000000000001</v>
       </c>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>70</v>
       </c>
@@ -2227,7 +2251,7 @@
         <v>6.8820000000000006</v>
       </c>
     </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>73</v>
       </c>
@@ -2248,7 +2272,7 @@
         <v>2.62</v>
       </c>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>76</v>
       </c>
@@ -2269,7 +2293,7 @@
         <v>4.7600000000000007</v>
       </c>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>81</v>
       </c>
@@ -2290,7 +2314,7 @@
         <v>3.81</v>
       </c>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>82</v>
       </c>
@@ -2311,7 +2335,7 @@
         <v>1.3320000000000001</v>
       </c>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>85</v>
       </c>
@@ -2332,7 +2356,7 @@
         <v>0.45800000000000002</v>
       </c>
     </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>90</v>
       </c>
@@ -2353,7 +2377,7 @@
         <v>2.6856</v>
       </c>
     </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>91</v>
       </c>
@@ -2374,7 +2398,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>95</v>
       </c>
@@ -2395,7 +2419,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>98</v>
       </c>
@@ -2416,7 +2440,7 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>102</v>
       </c>
@@ -2437,7 +2461,7 @@
         <v>0.36049999999999999</v>
       </c>
     </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>105</v>
       </c>
@@ -2458,7 +2482,7 @@
         <v>0.505</v>
       </c>
     </row>
-    <row r="33" spans="8:8" x14ac:dyDescent="0.45">
+    <row r="33" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H33" s="4"/>
     </row>
   </sheetData>
@@ -2495,14 +2519,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A84AF481-944A-4A4E-812B-EDDAA2A2EDA1}">
-  <dimension ref="A1:F7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.86328125" customWidth="1"/>
-    <col min="2" max="2" width="13.1328125" customWidth="1"/>
+    <col min="1" max="1" width="8.85546875" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>109</v>
       </c>
@@ -2512,15 +2536,18 @@
       <c r="C1" t="s">
         <v>31</v>
       </c>
-      <c r="E1" t="s">
+      <c r="D1" t="s">
+        <v>160</v>
+      </c>
+      <c r="F1" t="s">
         <v>115</v>
       </c>
-      <c r="F1" s="8">
+      <c r="G1" s="8">
         <f>SUM(C:C)</f>
-        <v>465.05000000000007</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+        <v>556.1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>110</v>
       </c>
@@ -2530,8 +2557,11 @@
       <c r="C2" s="4">
         <v>74.64</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="D2" s="4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>112</v>
       </c>
@@ -2541,8 +2571,11 @@
       <c r="C3" s="4">
         <v>6.98</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="D3" s="4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>113</v>
       </c>
@@ -2552,8 +2585,11 @@
       <c r="C4" s="4">
         <v>82.72</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="D4" s="4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>113</v>
       </c>
@@ -2563,8 +2599,11 @@
       <c r="C5" s="4">
         <v>48.95</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="D5" s="4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>112</v>
       </c>
@@ -2574,8 +2613,11 @@
       <c r="C6" s="4">
         <v>128.54</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="D6" s="4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>110</v>
       </c>
@@ -2584,6 +2626,66 @@
       </c>
       <c r="C7" s="4">
         <v>123.22</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>162</v>
+      </c>
+      <c r="B8" t="s">
+        <v>163</v>
+      </c>
+      <c r="C8" s="4">
+        <v>15.38</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>162</v>
+      </c>
+      <c r="B9" t="s">
+        <v>165</v>
+      </c>
+      <c r="C9" s="4">
+        <v>17.12</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>162</v>
+      </c>
+      <c r="B10" t="s">
+        <v>166</v>
+      </c>
+      <c r="C10" s="4">
+        <v>25.13</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>162</v>
+      </c>
+      <c r="B11" t="s">
+        <v>167</v>
+      </c>
+      <c r="C11" s="4">
+        <f>16.28+17.14</f>
+        <v>33.42</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
peripherals review and order
</commit_message>
<xml_diff>
--- a/part count estimates.xlsx
+++ b/part count estimates.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projects\computer\ax08\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc project\rlpc\AX08-PC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C39695F-9417-4CDC-B1F3-D23FC2D77ACA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A10F5BF-8811-401C-A90B-F42C908DDE87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="169">
   <si>
     <t>Register File</t>
   </si>
@@ -543,6 +543,9 @@
   </si>
   <si>
     <t>2 x Uart Adapter</t>
+  </si>
+  <si>
+    <t>peripherals</t>
   </si>
 </sst>
 </file>
@@ -653,9 +656,9 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Link" xfId="1" builtinId="8"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Währung" xfId="2" builtinId="4"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -934,16 +937,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P13"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" customWidth="1"/>
-    <col min="2" max="4" width="10.140625" customWidth="1"/>
-    <col min="7" max="8" width="10.140625" customWidth="1"/>
-    <col min="14" max="15" width="10.140625" customWidth="1"/>
-    <col min="16" max="16" width="48.28515625" customWidth="1"/>
+    <col min="1" max="1" width="17.86328125" customWidth="1"/>
+    <col min="2" max="4" width="10.1328125" customWidth="1"/>
+    <col min="7" max="8" width="10.1328125" customWidth="1"/>
+    <col min="14" max="15" width="10.1328125" customWidth="1"/>
+    <col min="16" max="16" width="48.265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.45">
       <c r="B1" t="s">
         <v>2</v>
       </c>
@@ -990,7 +993,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1037,7 +1040,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1084,7 +1087,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1131,7 +1134,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -1178,7 +1181,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -1225,7 +1228,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -1272,7 +1275,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1319,7 +1322,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -1366,7 +1369,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -1413,7 +1416,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1463,7 +1466,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>39</v>
       </c>
@@ -1532,14 +1535,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1780C73-0264-4CD0-A807-67CE58F9B4CA}">
   <dimension ref="A1:D36"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3984375" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="16.5703125" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="16.59765625" customWidth="1"/>
+    <col min="3" max="3" width="12.73046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>129</v>
       </c>
@@ -1553,7 +1556,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B2" t="s">
         <v>116</v>
       </c>
@@ -1564,7 +1567,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B3" t="s">
         <v>146</v>
       </c>
@@ -1575,7 +1578,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B4" t="s">
         <v>119</v>
       </c>
@@ -1586,7 +1589,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B5" t="s">
         <v>143</v>
       </c>
@@ -1597,7 +1600,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
         <v>120</v>
       </c>
@@ -1608,7 +1611,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B7" t="s">
         <v>121</v>
       </c>
@@ -1619,7 +1622,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>123</v>
       </c>
@@ -1633,7 +1636,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
         <v>116</v>
       </c>
@@ -1644,7 +1647,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
         <v>119</v>
       </c>
@@ -1655,7 +1658,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
         <v>143</v>
       </c>
@@ -1666,7 +1669,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B13" t="s">
         <v>120</v>
       </c>
@@ -1677,7 +1680,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>130</v>
       </c>
@@ -1691,7 +1694,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B16" t="s">
         <v>116</v>
       </c>
@@ -1702,7 +1705,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B17" t="s">
         <v>119</v>
       </c>
@@ -1713,7 +1716,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B18" t="s">
         <v>143</v>
       </c>
@@ -1724,7 +1727,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B19" t="s">
         <v>120</v>
       </c>
@@ -1735,7 +1738,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B20" t="s">
         <v>133</v>
       </c>
@@ -1746,7 +1749,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B21" t="s">
         <v>134</v>
       </c>
@@ -1757,7 +1760,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>135</v>
       </c>
@@ -1771,7 +1774,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B24" t="s">
         <v>153</v>
       </c>
@@ -1782,7 +1785,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B25" t="s">
         <v>150</v>
       </c>
@@ -1793,7 +1796,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B26" t="s">
         <v>154</v>
       </c>
@@ -1804,7 +1807,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B27" t="s">
         <v>155</v>
       </c>
@@ -1815,7 +1818,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B28" t="s">
         <v>156</v>
       </c>
@@ -1826,7 +1829,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>136</v>
       </c>
@@ -1840,7 +1843,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B31" t="s">
         <v>120</v>
       </c>
@@ -1851,7 +1854,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B32" t="s">
         <v>67</v>
       </c>
@@ -1862,7 +1865,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="33" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B33" t="s">
         <v>66</v>
       </c>
@@ -1873,7 +1876,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="34" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B34" t="s">
         <v>137</v>
       </c>
@@ -1884,7 +1887,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="35" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B35" t="s">
         <v>138</v>
       </c>
@@ -1895,7 +1898,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="36" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B36" t="s">
         <v>139</v>
       </c>
@@ -1914,14 +1917,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A2F25C3-A040-4D55-A5F0-DFC308DB6F13}">
   <dimension ref="B1:K33"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="29.7109375" customWidth="1"/>
-    <col min="6" max="6" width="109.7109375" customWidth="1"/>
+    <col min="2" max="2" width="26.86328125" customWidth="1"/>
+    <col min="3" max="3" width="29.73046875" customWidth="1"/>
+    <col min="6" max="6" width="109.73046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:11" x14ac:dyDescent="0.45">
       <c r="H1" t="s">
         <v>35</v>
       </c>
@@ -1933,14 +1936,14 @@
         <v>10.8</v>
       </c>
     </row>
-    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.45">
       <c r="H2" s="4">
         <f>SUM(H5:H996)</f>
         <v>123.93560000000001</v>
       </c>
     </row>
-    <row r="3" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="4" spans="2:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B4" s="5" t="s">
         <v>28</v>
       </c>
@@ -1959,7 +1962,7 @@
       <c r="G4" s="6"/>
       <c r="H4" s="7"/>
     </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B5" t="s">
         <v>34</v>
       </c>
@@ -1981,7 +1984,7 @@
         <v>21.6</v>
       </c>
     </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
         <v>37</v>
       </c>
@@ -1999,7 +2002,7 @@
         <v>40.599999999999994</v>
       </c>
     </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B7" t="s">
         <v>40</v>
       </c>
@@ -2020,7 +2023,7 @@
         <v>17.335999999999999</v>
       </c>
     </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
         <v>43</v>
       </c>
@@ -2041,7 +2044,7 @@
         <v>7.645999999999999</v>
       </c>
     </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
         <v>44</v>
       </c>
@@ -2062,7 +2065,7 @@
         <v>2.7639999999999998</v>
       </c>
     </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
         <v>46</v>
       </c>
@@ -2083,7 +2086,7 @@
         <v>1.2089999999999999</v>
       </c>
     </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
         <v>51</v>
       </c>
@@ -2104,7 +2107,7 @@
         <v>0.75050000000000006</v>
       </c>
     </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
         <v>48</v>
       </c>
@@ -2125,7 +2128,7 @@
         <v>0.9355</v>
       </c>
     </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B13" t="s">
         <v>53</v>
       </c>
@@ -2146,7 +2149,7 @@
         <v>0.85450000000000004</v>
       </c>
     </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B14" t="s">
         <v>55</v>
       </c>
@@ -2167,7 +2170,7 @@
         <v>0.7679999999999999</v>
       </c>
     </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B15" t="s">
         <v>57</v>
       </c>
@@ -2188,7 +2191,7 @@
         <v>1.099</v>
       </c>
     </row>
-    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B16" t="s">
         <v>59</v>
       </c>
@@ -2209,7 +2212,7 @@
         <v>0.89899999999999991</v>
       </c>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B17" t="s">
         <v>108</v>
       </c>
@@ -2230,7 +2233,7 @@
         <v>2.0110000000000001</v>
       </c>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B18" t="s">
         <v>70</v>
       </c>
@@ -2251,7 +2254,7 @@
         <v>6.8820000000000006</v>
       </c>
     </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B19" t="s">
         <v>73</v>
       </c>
@@ -2272,7 +2275,7 @@
         <v>2.62</v>
       </c>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B20" t="s">
         <v>76</v>
       </c>
@@ -2293,7 +2296,7 @@
         <v>4.7600000000000007</v>
       </c>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B21" t="s">
         <v>81</v>
       </c>
@@ -2314,7 +2317,7 @@
         <v>3.81</v>
       </c>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B22" t="s">
         <v>82</v>
       </c>
@@ -2335,7 +2338,7 @@
         <v>1.3320000000000001</v>
       </c>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B23" t="s">
         <v>85</v>
       </c>
@@ -2356,7 +2359,7 @@
         <v>0.45800000000000002</v>
       </c>
     </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B24" t="s">
         <v>90</v>
       </c>
@@ -2377,7 +2380,7 @@
         <v>2.6856</v>
       </c>
     </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B25" t="s">
         <v>91</v>
       </c>
@@ -2398,7 +2401,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B26" t="s">
         <v>95</v>
       </c>
@@ -2419,7 +2422,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B27" t="s">
         <v>98</v>
       </c>
@@ -2440,7 +2443,7 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B28" t="s">
         <v>102</v>
       </c>
@@ -2461,7 +2464,7 @@
         <v>0.36049999999999999</v>
       </c>
     </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B29" t="s">
         <v>105</v>
       </c>
@@ -2482,7 +2485,7 @@
         <v>0.505</v>
       </c>
     </row>
-    <row r="33" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="8:8" x14ac:dyDescent="0.45">
       <c r="H33" s="4"/>
     </row>
   </sheetData>
@@ -2519,14 +2522,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A84AF481-944A-4A4E-812B-EDDAA2A2EDA1}">
-  <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="8.85546875" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" customWidth="1"/>
+    <col min="1" max="1" width="8.86328125" customWidth="1"/>
+    <col min="2" max="2" width="13.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>109</v>
       </c>
@@ -2544,10 +2547,10 @@
       </c>
       <c r="G1" s="8">
         <f>SUM(C:C)</f>
-        <v>556.1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>569.34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>110</v>
       </c>
@@ -2561,7 +2564,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>112</v>
       </c>
@@ -2575,7 +2578,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>113</v>
       </c>
@@ -2589,7 +2592,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>113</v>
       </c>
@@ -2603,7 +2606,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>112</v>
       </c>
@@ -2617,7 +2620,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>110</v>
       </c>
@@ -2631,7 +2634,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>162</v>
       </c>
@@ -2645,7 +2648,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>162</v>
       </c>
@@ -2659,7 +2662,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>162</v>
       </c>
@@ -2673,7 +2676,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>162</v>
       </c>
@@ -2686,6 +2689,20 @@
       </c>
       <c r="D11" s="4" t="s">
         <v>164</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>112</v>
+      </c>
+      <c r="B12" t="s">
+        <v>168</v>
+      </c>
+      <c r="C12" s="4">
+        <v>13.24</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ax08 main review and order
</commit_message>
<xml_diff>
--- a/part count estimates.xlsx
+++ b/part count estimates.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc project\rlpc\AX08-PC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc_project\rlpc\AX08-PC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A10F5BF-8811-401C-A90B-F42C908DDE87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC71D22B-9BA4-4455-875E-0E6F6AF2E29C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="170">
   <si>
     <t>Register File</t>
   </si>
@@ -546,6 +546,9 @@
   </si>
   <si>
     <t>peripherals</t>
+  </si>
+  <si>
+    <t>main</t>
   </si>
 </sst>
 </file>
@@ -2522,7 +2525,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A84AF481-944A-4A4E-812B-EDDAA2A2EDA1}">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="8.86328125" customWidth="1"/>
@@ -2547,7 +2550,7 @@
       </c>
       <c r="G1" s="8">
         <f>SUM(C:C)</f>
-        <v>569.34</v>
+        <v>711.19</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.45">
@@ -2702,6 +2705,20 @@
         <v>13.24</v>
       </c>
       <c r="D12" s="4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>112</v>
+      </c>
+      <c r="B13" t="s">
+        <v>169</v>
+      </c>
+      <c r="C13" s="4">
+        <v>141.85</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>161</v>
       </c>
     </row>

</xml_diff>

<commit_message>
finalized orders 1 tab
</commit_message>
<xml_diff>
--- a/part count estimates.xlsx
+++ b/part count estimates.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc_project\rlpc\AX08-PC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E739B05-E138-4909-8BB3-8F1EB2838027}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41289F45-D7C8-4994-8A01-7BBD889BD2C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,8 @@
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
     <sheet name="notes" sheetId="5" r:id="rId2"/>
     <sheet name="part_links" sheetId="3" r:id="rId3"/>
-    <sheet name="orders" sheetId="4" r:id="rId4"/>
+    <sheet name="orders" sheetId="6" r:id="rId4"/>
+    <sheet name="orders 1" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="174">
   <si>
     <t>Register File</t>
   </si>
@@ -552,6 +553,15 @@
   </si>
   <si>
     <t>frontpanel</t>
+  </si>
+  <si>
+    <t>Oliver:</t>
+  </si>
+  <si>
+    <t>Peter:</t>
+  </si>
+  <si>
+    <t>open:</t>
   </si>
 </sst>
 </file>
@@ -646,7 +656,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -660,6 +670,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -2527,6 +2538,118 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E557F82-F62A-41C0-9A94-AB7F3EDBF023}">
+  <dimension ref="A1:G15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="8.86328125" customWidth="1"/>
+    <col min="2" max="2" width="13.1328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" t="s">
+        <v>160</v>
+      </c>
+      <c r="F1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G1" s="8">
+        <f>SUM(C:C)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="F2" t="s">
+        <v>171</v>
+      </c>
+      <c r="G2" s="8">
+        <f>SUMIFS(C:C,D:D,"Oliver")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="F3" t="s">
+        <v>172</v>
+      </c>
+      <c r="G3" s="8">
+        <f>SUMIFS(C:C,D:D,"Peter")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="F4" t="s">
+        <v>173</v>
+      </c>
+      <c r="G4" s="9">
+        <f>(G2-G3)/2</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A84AF481-944A-4A4E-812B-EDDAA2A2EDA1}">
   <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -2569,6 +2692,13 @@
       <c r="D2" s="4" t="s">
         <v>161</v>
       </c>
+      <c r="F2" t="s">
+        <v>171</v>
+      </c>
+      <c r="G2" s="8">
+        <f>SUMIFS(C:C,D:D,"Oliver")</f>
+        <v>656.8900000000001</v>
+      </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
@@ -2583,6 +2713,13 @@
       <c r="D3" s="4" t="s">
         <v>161</v>
       </c>
+      <c r="F3" t="s">
+        <v>172</v>
+      </c>
+      <c r="G3" s="8">
+        <f>SUMIFS(C:C,D:D,"Peter")</f>
+        <v>91.05</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
@@ -2596,6 +2733,13 @@
       </c>
       <c r="D4" s="4" t="s">
         <v>161</v>
+      </c>
+      <c r="F4" t="s">
+        <v>173</v>
+      </c>
+      <c r="G4" s="9">
+        <f>(G2-G3)/2</f>
+        <v>282.92000000000007</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.45">

</xml_diff>